<commit_message>
Daily price update - 2026-10-09
</commit_message>
<xml_diff>
--- a/flight_prices.xlsx
+++ b/flight_prices.xlsx
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-10-08 15:13</t>
+          <t>Last updated: 2026-10-09 14:58</t>
         </is>
       </c>
     </row>
@@ -664,10 +664,10 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>140</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G274"/>
+  <dimension ref="A1:G280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15621,151 +15621,92 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" ht="18" customHeight="1">
-      <c r="A127" s="11" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B126" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="G126" s="17" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="128" ht="18" customHeight="1">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 20:30_AIR_ret_AIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B129" s="12" t="inlineStr">
+        <is>
+          <t>20:30_AIR_ret_AIR</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>Air France</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>Air France</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="n">
+        <v>547</v>
+      </c>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="18" customHeight="1">
+      <c r="A131" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Combination: 21:30_IBE_ret_IBE</t>
         </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="B128" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D128" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E128" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F128" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="G128" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="B129" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D129" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E129" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F129" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="G129" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="B130" s="12" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C130" s="5" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D130" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E130" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F130" s="6" t="n">
-        <v>206</v>
-      </c>
-      <c r="G130" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="B131" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="C131" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D131" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E131" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="F131" s="9" t="n">
-        <v>206</v>
-      </c>
-      <c r="G131" s="14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B132" s="12" t="inlineStr">
@@ -15791,14 +15732,16 @@
       <c r="F132" s="6" t="n">
         <v>206</v>
       </c>
-      <c r="G132" s="15" t="n">
-        <v>0</v>
+      <c r="G132" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B133" s="13" t="inlineStr">
@@ -15822,16 +15765,16 @@
         </is>
       </c>
       <c r="F133" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G133" s="16" t="n">
-        <v>7</v>
+        <v>206</v>
+      </c>
+      <c r="G133" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B134" s="12" t="inlineStr">
@@ -15855,7 +15798,7 @@
         </is>
       </c>
       <c r="F134" s="6" t="n">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="G134" s="15" t="n">
         <v>0</v>
@@ -15864,7 +15807,7 @@
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B135" s="13" t="inlineStr">
@@ -15888,7 +15831,7 @@
         </is>
       </c>
       <c r="F135" s="9" t="n">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="G135" s="14" t="n">
         <v>0</v>
@@ -15897,7 +15840,7 @@
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B136" s="12" t="inlineStr">
@@ -15921,7 +15864,7 @@
         </is>
       </c>
       <c r="F136" s="6" t="n">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="G136" s="15" t="n">
         <v>0</v>
@@ -15930,7 +15873,7 @@
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B137" s="13" t="inlineStr">
@@ -15956,14 +15899,14 @@
       <c r="F137" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="G137" s="14" t="n">
-        <v>0</v>
+      <c r="G137" s="16" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B138" s="12" t="inlineStr">
@@ -15996,7 +15939,7 @@
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B139" s="13" t="inlineStr">
@@ -16029,7 +15972,7 @@
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B140" s="12" t="inlineStr">
@@ -16053,16 +15996,16 @@
         </is>
       </c>
       <c r="F140" s="6" t="n">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="G140" s="15" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="8" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B141" s="13" t="inlineStr">
@@ -16086,7 +16029,7 @@
         </is>
       </c>
       <c r="F141" s="9" t="n">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="G141" s="14" t="n">
         <v>0</v>
@@ -16095,7 +16038,7 @@
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B142" s="12" t="inlineStr">
@@ -16119,7 +16062,7 @@
         </is>
       </c>
       <c r="F142" s="6" t="n">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="G142" s="15" t="n">
         <v>0</v>
@@ -16128,7 +16071,7 @@
     <row r="143">
       <c r="A143" s="8" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B143" s="13" t="inlineStr">
@@ -16152,7 +16095,7 @@
         </is>
       </c>
       <c r="F143" s="9" t="n">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="G143" s="14" t="n">
         <v>0</v>
@@ -16161,7 +16104,7 @@
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B144" s="12" t="inlineStr">
@@ -16188,13 +16131,13 @@
         <v>206</v>
       </c>
       <c r="G144" s="15" t="n">
-        <v>0</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B145" s="13" t="inlineStr">
@@ -16227,7 +16170,7 @@
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B146" s="12" t="inlineStr">
@@ -16260,7 +16203,7 @@
     <row r="147">
       <c r="A147" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B147" s="13" t="inlineStr">
@@ -16293,7 +16236,7 @@
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B148" s="12" t="inlineStr">
@@ -16326,7 +16269,7 @@
     <row r="149">
       <c r="A149" s="8" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B149" s="13" t="inlineStr">
@@ -16359,7 +16302,7 @@
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B150" s="12" t="inlineStr">
@@ -16383,16 +16326,16 @@
         </is>
       </c>
       <c r="F150" s="6" t="n">
-        <v>227</v>
-      </c>
-      <c r="G150" s="17" t="n">
-        <v>21</v>
+        <v>206</v>
+      </c>
+      <c r="G150" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="8" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B151" s="13" t="inlineStr">
@@ -16416,7 +16359,7 @@
         </is>
       </c>
       <c r="F151" s="9" t="n">
-        <v>227</v>
+        <v>206</v>
       </c>
       <c r="G151" s="14" t="n">
         <v>0</v>
@@ -16425,7 +16368,7 @@
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B152" s="12" t="inlineStr">
@@ -16449,7 +16392,7 @@
         </is>
       </c>
       <c r="F152" s="6" t="n">
-        <v>227</v>
+        <v>206</v>
       </c>
       <c r="G152" s="15" t="n">
         <v>0</v>
@@ -16458,7 +16401,7 @@
     <row r="153">
       <c r="A153" s="8" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B153" s="13" t="inlineStr">
@@ -16482,7 +16425,7 @@
         </is>
       </c>
       <c r="F153" s="9" t="n">
-        <v>227</v>
+        <v>206</v>
       </c>
       <c r="G153" s="14" t="n">
         <v>0</v>
@@ -16491,7 +16434,7 @@
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B154" s="12" t="inlineStr">
@@ -16517,14 +16460,14 @@
       <c r="F154" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="G154" s="15" t="n">
-        <v>0</v>
+      <c r="G154" s="17" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B155" s="13" t="inlineStr">
@@ -16557,7 +16500,7 @@
     <row r="156">
       <c r="A156" s="5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B156" s="12" t="inlineStr">
@@ -16590,7 +16533,7 @@
     <row r="157">
       <c r="A157" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B157" s="13" t="inlineStr">
@@ -16623,7 +16566,7 @@
     <row r="158">
       <c r="A158" s="5" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B158" s="12" t="inlineStr">
@@ -16656,7 +16599,7 @@
     <row r="159">
       <c r="A159" s="8" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B159" s="13" t="inlineStr">
@@ -16689,7 +16632,7 @@
     <row r="160">
       <c r="A160" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B160" s="12" t="inlineStr">
@@ -16722,7 +16665,7 @@
     <row r="161">
       <c r="A161" s="8" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B161" s="13" t="inlineStr">
@@ -16755,7 +16698,7 @@
     <row r="162">
       <c r="A162" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B162" s="12" t="inlineStr">
@@ -16788,7 +16731,7 @@
     <row r="163">
       <c r="A163" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B163" s="13" t="inlineStr">
@@ -16821,7 +16764,7 @@
     <row r="164">
       <c r="A164" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B164" s="12" t="inlineStr">
@@ -16854,7 +16797,7 @@
     <row r="165">
       <c r="A165" s="8" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B165" s="13" t="inlineStr">
@@ -16887,7 +16830,7 @@
     <row r="166">
       <c r="A166" s="5" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B166" s="12" t="inlineStr">
@@ -16920,7 +16863,7 @@
     <row r="167">
       <c r="A167" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B167" s="13" t="inlineStr">
@@ -16953,7 +16896,7 @@
     <row r="168">
       <c r="A168" s="5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B168" s="12" t="inlineStr">
@@ -16986,7 +16929,7 @@
     <row r="169">
       <c r="A169" s="8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B169" s="13" t="inlineStr">
@@ -17019,7 +16962,7 @@
     <row r="170">
       <c r="A170" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B170" s="12" t="inlineStr">
@@ -17052,7 +16995,7 @@
     <row r="171">
       <c r="A171" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B171" s="13" t="inlineStr">
@@ -17085,7 +17028,7 @@
     <row r="172">
       <c r="A172" s="5" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B172" s="12" t="inlineStr">
@@ -17118,7 +17061,7 @@
     <row r="173">
       <c r="A173" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B173" s="13" t="inlineStr">
@@ -17151,7 +17094,7 @@
     <row r="174">
       <c r="A174" s="5" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B174" s="12" t="inlineStr">
@@ -17184,7 +17127,7 @@
     <row r="175">
       <c r="A175" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B175" s="13" t="inlineStr">
@@ -17217,7 +17160,7 @@
     <row r="176">
       <c r="A176" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B176" s="12" t="inlineStr">
@@ -17241,16 +17184,16 @@
         </is>
       </c>
       <c r="F176" s="6" t="n">
-        <v>237</v>
-      </c>
-      <c r="G176" s="17" t="n">
-        <v>10</v>
+        <v>227</v>
+      </c>
+      <c r="G176" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B177" s="13" t="inlineStr">
@@ -17274,16 +17217,16 @@
         </is>
       </c>
       <c r="F177" s="9" t="n">
-        <v>246</v>
-      </c>
-      <c r="G177" s="16" t="n">
-        <v>9</v>
+        <v>227</v>
+      </c>
+      <c r="G177" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B178" s="12" t="inlineStr">
@@ -17307,7 +17250,7 @@
         </is>
       </c>
       <c r="F178" s="6" t="n">
-        <v>246</v>
+        <v>227</v>
       </c>
       <c r="G178" s="15" t="n">
         <v>0</v>
@@ -17316,7 +17259,7 @@
     <row r="179">
       <c r="A179" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B179" s="13" t="inlineStr">
@@ -17340,7 +17283,7 @@
         </is>
       </c>
       <c r="F179" s="9" t="n">
-        <v>246</v>
+        <v>227</v>
       </c>
       <c r="G179" s="14" t="n">
         <v>0</v>
@@ -17349,7 +17292,7 @@
     <row r="180">
       <c r="A180" s="5" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B180" s="12" t="inlineStr">
@@ -17373,16 +17316,16 @@
         </is>
       </c>
       <c r="F180" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="G180" s="15" t="n">
-        <v>0</v>
+        <v>237</v>
+      </c>
+      <c r="G180" s="17" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B181" s="13" t="inlineStr">
@@ -17408,14 +17351,14 @@
       <c r="F181" s="9" t="n">
         <v>246</v>
       </c>
-      <c r="G181" s="14" t="n">
-        <v>0</v>
+      <c r="G181" s="16" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="5" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B182" s="12" t="inlineStr">
@@ -17448,7 +17391,7 @@
     <row r="183">
       <c r="A183" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B183" s="13" t="inlineStr">
@@ -17481,7 +17424,7 @@
     <row r="184">
       <c r="A184" s="5" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B184" s="12" t="inlineStr">
@@ -17505,16 +17448,16 @@
         </is>
       </c>
       <c r="F184" s="6" t="n">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G184" s="15" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B185" s="13" t="inlineStr">
@@ -17540,14 +17483,14 @@
       <c r="F185" s="9" t="n">
         <v>246</v>
       </c>
-      <c r="G185" s="16" t="n">
-        <v>2</v>
+      <c r="G185" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B186" s="12" t="inlineStr">
@@ -17580,7 +17523,7 @@
     <row r="187">
       <c r="A187" s="8" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B187" s="13" t="inlineStr">
@@ -17613,7 +17556,7 @@
     <row r="188">
       <c r="A188" s="5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B188" s="12" t="inlineStr">
@@ -17637,16 +17580,16 @@
         </is>
       </c>
       <c r="F188" s="6" t="n">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="G188" s="15" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B189" s="13" t="inlineStr">
@@ -17672,14 +17615,14 @@
       <c r="F189" s="9" t="n">
         <v>246</v>
       </c>
-      <c r="G189" s="14" t="n">
-        <v>0</v>
+      <c r="G189" s="16" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="5" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B190" s="12" t="inlineStr">
@@ -17712,7 +17655,7 @@
     <row r="191">
       <c r="A191" s="8" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B191" s="13" t="inlineStr">
@@ -17745,7 +17688,7 @@
     <row r="192">
       <c r="A192" s="5" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B192" s="12" t="inlineStr">
@@ -17778,7 +17721,7 @@
     <row r="193">
       <c r="A193" s="8" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B193" s="13" t="inlineStr">
@@ -17811,7 +17754,7 @@
     <row r="194">
       <c r="A194" s="5" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B194" s="12" t="inlineStr">
@@ -17844,7 +17787,7 @@
     <row r="195">
       <c r="A195" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B195" s="13" t="inlineStr">
@@ -17877,7 +17820,7 @@
     <row r="196">
       <c r="A196" s="5" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B196" s="12" t="inlineStr">
@@ -17910,7 +17853,7 @@
     <row r="197">
       <c r="A197" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B197" s="13" t="inlineStr">
@@ -17943,7 +17886,7 @@
     <row r="198">
       <c r="A198" s="5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B198" s="12" t="inlineStr">
@@ -17976,7 +17919,7 @@
     <row r="199">
       <c r="A199" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B199" s="13" t="inlineStr">
@@ -18000,16 +17943,16 @@
         </is>
       </c>
       <c r="F199" s="9" t="n">
-        <v>255</v>
-      </c>
-      <c r="G199" s="16" t="n">
-        <v>9</v>
+        <v>246</v>
+      </c>
+      <c r="G199" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="5" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B200" s="12" t="inlineStr">
@@ -18033,7 +17976,7 @@
         </is>
       </c>
       <c r="F200" s="6" t="n">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="G200" s="15" t="n">
         <v>0</v>
@@ -18042,7 +17985,7 @@
     <row r="201">
       <c r="A201" s="8" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B201" s="13" t="inlineStr">
@@ -18066,7 +18009,7 @@
         </is>
       </c>
       <c r="F201" s="9" t="n">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="G201" s="14" t="n">
         <v>0</v>
@@ -18075,7 +18018,7 @@
     <row r="202">
       <c r="A202" s="5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B202" s="12" t="inlineStr">
@@ -18099,7 +18042,7 @@
         </is>
       </c>
       <c r="F202" s="6" t="n">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="G202" s="15" t="n">
         <v>0</v>
@@ -18108,7 +18051,7 @@
     <row r="203">
       <c r="A203" s="8" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B203" s="13" t="inlineStr">
@@ -18132,16 +18075,16 @@
         </is>
       </c>
       <c r="F203" s="9" t="n">
-        <v>180</v>
-      </c>
-      <c r="G203" s="14" t="n">
-        <v>-75</v>
+        <v>255</v>
+      </c>
+      <c r="G203" s="16" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="5" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B204" s="12" t="inlineStr">
@@ -18165,7 +18108,7 @@
         </is>
       </c>
       <c r="F204" s="6" t="n">
-        <v>180</v>
+        <v>255</v>
       </c>
       <c r="G204" s="15" t="n">
         <v>0</v>
@@ -18174,7 +18117,7 @@
     <row r="205">
       <c r="A205" s="8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B205" s="13" t="inlineStr">
@@ -18198,7 +18141,7 @@
         </is>
       </c>
       <c r="F205" s="9" t="n">
-        <v>180</v>
+        <v>255</v>
       </c>
       <c r="G205" s="14" t="n">
         <v>0</v>
@@ -18207,7 +18150,7 @@
     <row r="206">
       <c r="A206" s="5" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B206" s="12" t="inlineStr">
@@ -18231,7 +18174,7 @@
         </is>
       </c>
       <c r="F206" s="6" t="n">
-        <v>180</v>
+        <v>255</v>
       </c>
       <c r="G206" s="15" t="n">
         <v>0</v>
@@ -18240,7 +18183,7 @@
     <row r="207">
       <c r="A207" s="8" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B207" s="13" t="inlineStr">
@@ -18267,13 +18210,13 @@
         <v>180</v>
       </c>
       <c r="G207" s="14" t="n">
-        <v>0</v>
+        <v>-75</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="5" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B208" s="12" t="inlineStr">
@@ -18306,7 +18249,7 @@
     <row r="209">
       <c r="A209" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B209" s="13" t="inlineStr">
@@ -18339,7 +18282,7 @@
     <row r="210">
       <c r="A210" s="5" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B210" s="12" t="inlineStr">
@@ -18363,16 +18306,16 @@
         </is>
       </c>
       <c r="F210" s="6" t="n">
-        <v>199</v>
-      </c>
-      <c r="G210" s="17" t="n">
-        <v>19</v>
+        <v>180</v>
+      </c>
+      <c r="G210" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="8" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B211" s="13" t="inlineStr">
@@ -18396,16 +18339,16 @@
         </is>
       </c>
       <c r="F211" s="9" t="n">
-        <v>211</v>
-      </c>
-      <c r="G211" s="16" t="n">
-        <v>12</v>
+        <v>180</v>
+      </c>
+      <c r="G211" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B212" s="12" t="inlineStr">
@@ -18429,16 +18372,16 @@
         </is>
       </c>
       <c r="F212" s="6" t="n">
-        <v>216</v>
-      </c>
-      <c r="G212" s="17" t="n">
-        <v>5</v>
+        <v>180</v>
+      </c>
+      <c r="G212" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="8" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B213" s="13" t="inlineStr">
@@ -18462,16 +18405,16 @@
         </is>
       </c>
       <c r="F213" s="9" t="n">
-        <v>228</v>
-      </c>
-      <c r="G213" s="16" t="n">
-        <v>12</v>
+        <v>180</v>
+      </c>
+      <c r="G213" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B214" s="12" t="inlineStr">
@@ -18495,16 +18438,16 @@
         </is>
       </c>
       <c r="F214" s="6" t="n">
-        <v>228</v>
-      </c>
-      <c r="G214" s="15" t="n">
-        <v>0</v>
+        <v>199</v>
+      </c>
+      <c r="G214" s="17" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="8" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B215" s="13" t="inlineStr">
@@ -18528,16 +18471,16 @@
         </is>
       </c>
       <c r="F215" s="9" t="n">
-        <v>228</v>
-      </c>
-      <c r="G215" s="14" t="n">
-        <v>0</v>
+        <v>211</v>
+      </c>
+      <c r="G215" s="16" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B216" s="12" t="inlineStr">
@@ -18561,7 +18504,7 @@
         </is>
       </c>
       <c r="F216" s="6" t="n">
-        <v>233</v>
+        <v>216</v>
       </c>
       <c r="G216" s="17" t="n">
         <v>5</v>
@@ -18570,7 +18513,7 @@
     <row r="217">
       <c r="A217" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B217" s="13" t="inlineStr">
@@ -18594,16 +18537,16 @@
         </is>
       </c>
       <c r="F217" s="9" t="n">
-        <v>233</v>
-      </c>
-      <c r="G217" s="14" t="n">
-        <v>0</v>
+        <v>228</v>
+      </c>
+      <c r="G217" s="16" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B218" s="12" t="inlineStr">
@@ -18627,7 +18570,7 @@
         </is>
       </c>
       <c r="F218" s="6" t="n">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="G218" s="15" t="n">
         <v>0</v>
@@ -18636,7 +18579,7 @@
     <row r="219">
       <c r="A219" s="8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B219" s="13" t="inlineStr">
@@ -18660,7 +18603,7 @@
         </is>
       </c>
       <c r="F219" s="9" t="n">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="G219" s="14" t="n">
         <v>0</v>
@@ -18669,7 +18612,7 @@
     <row r="220">
       <c r="A220" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B220" s="12" t="inlineStr">
@@ -18695,14 +18638,14 @@
       <c r="F220" s="6" t="n">
         <v>233</v>
       </c>
-      <c r="G220" s="15" t="n">
-        <v>0</v>
+      <c r="G220" s="17" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="8" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B221" s="13" t="inlineStr">
@@ -18735,7 +18678,7 @@
     <row r="222">
       <c r="A222" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B222" s="12" t="inlineStr">
@@ -18768,7 +18711,7 @@
     <row r="223">
       <c r="A223" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B223" s="13" t="inlineStr">
@@ -18801,7 +18744,7 @@
     <row r="224">
       <c r="A224" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B224" s="12" t="inlineStr">
@@ -18825,16 +18768,16 @@
         </is>
       </c>
       <c r="F224" s="6" t="n">
-        <v>239</v>
-      </c>
-      <c r="G224" s="17" t="n">
-        <v>6</v>
+        <v>233</v>
+      </c>
+      <c r="G224" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B225" s="13" t="inlineStr">
@@ -18861,13 +18804,13 @@
         <v>233</v>
       </c>
       <c r="G225" s="14" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B226" s="12" t="inlineStr">
@@ -18900,7 +18843,7 @@
     <row r="227">
       <c r="A227" s="8" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B227" s="13" t="inlineStr">
@@ -18924,16 +18867,16 @@
         </is>
       </c>
       <c r="F227" s="9" t="n">
-        <v>239</v>
-      </c>
-      <c r="G227" s="16" t="n">
-        <v>6</v>
+        <v>233</v>
+      </c>
+      <c r="G227" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B228" s="12" t="inlineStr">
@@ -18959,14 +18902,14 @@
       <c r="F228" s="6" t="n">
         <v>239</v>
       </c>
-      <c r="G228" s="15" t="n">
-        <v>0</v>
+      <c r="G228" s="17" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B229" s="13" t="inlineStr">
@@ -18990,16 +18933,16 @@
         </is>
       </c>
       <c r="F229" s="9" t="n">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="G229" s="14" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B230" s="12" t="inlineStr">
@@ -19023,7 +18966,7 @@
         </is>
       </c>
       <c r="F230" s="6" t="n">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="G230" s="15" t="n">
         <v>0</v>
@@ -19032,7 +18975,7 @@
     <row r="231">
       <c r="A231" s="8" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B231" s="13" t="inlineStr">
@@ -19056,16 +18999,16 @@
         </is>
       </c>
       <c r="F231" s="9" t="n">
-        <v>256</v>
+        <v>239</v>
       </c>
       <c r="G231" s="16" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B232" s="12" t="inlineStr">
@@ -19089,16 +19032,16 @@
         </is>
       </c>
       <c r="F232" s="6" t="n">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="G232" s="15" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B233" s="13" t="inlineStr">
@@ -19122,7 +19065,7 @@
         </is>
       </c>
       <c r="F233" s="9" t="n">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="G233" s="14" t="n">
         <v>0</v>
@@ -19131,7 +19074,7 @@
     <row r="234">
       <c r="A234" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B234" s="12" t="inlineStr">
@@ -19155,16 +19098,16 @@
         </is>
       </c>
       <c r="F234" s="6" t="n">
-        <v>160</v>
+        <v>239</v>
       </c>
       <c r="G234" s="15" t="n">
-        <v>-91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="8" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B235" s="13" t="inlineStr">
@@ -19188,16 +19131,16 @@
         </is>
       </c>
       <c r="F235" s="9" t="n">
-        <v>166</v>
+        <v>256</v>
       </c>
       <c r="G235" s="16" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B236" s="12" t="inlineStr">
@@ -19221,16 +19164,16 @@
         </is>
       </c>
       <c r="F236" s="6" t="n">
-        <v>185</v>
-      </c>
-      <c r="G236" s="17" t="n">
-        <v>19</v>
+        <v>251</v>
+      </c>
+      <c r="G236" s="15" t="n">
+        <v>-5</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B237" s="13" t="inlineStr">
@@ -19254,7 +19197,7 @@
         </is>
       </c>
       <c r="F237" s="9" t="n">
-        <v>185</v>
+        <v>251</v>
       </c>
       <c r="G237" s="14" t="n">
         <v>0</v>
@@ -19263,7 +19206,7 @@
     <row r="238">
       <c r="A238" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B238" s="12" t="inlineStr">
@@ -19287,16 +19230,16 @@
         </is>
       </c>
       <c r="F238" s="6" t="n">
-        <v>185</v>
+        <v>160</v>
       </c>
       <c r="G238" s="15" t="n">
-        <v>0</v>
+        <v>-91</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B239" s="13" t="inlineStr">
@@ -19320,7 +19263,7 @@
         </is>
       </c>
       <c r="F239" s="9" t="n">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="G239" s="16" t="n">
         <v>6</v>
@@ -19329,7 +19272,7 @@
     <row r="240">
       <c r="A240" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B240" s="12" t="inlineStr">
@@ -19353,16 +19296,16 @@
         </is>
       </c>
       <c r="F240" s="6" t="n">
-        <v>191</v>
-      </c>
-      <c r="G240" s="15" t="n">
-        <v>0</v>
+        <v>185</v>
+      </c>
+      <c r="G240" s="17" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B241" s="13" t="inlineStr">
@@ -19386,7 +19329,7 @@
         </is>
       </c>
       <c r="F241" s="9" t="n">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="G241" s="14" t="n">
         <v>0</v>
@@ -19395,7 +19338,7 @@
     <row r="242">
       <c r="A242" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B242" s="12" t="inlineStr">
@@ -19419,7 +19362,7 @@
         </is>
       </c>
       <c r="F242" s="6" t="n">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="G242" s="15" t="n">
         <v>0</v>
@@ -19428,7 +19371,7 @@
     <row r="243">
       <c r="A243" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B243" s="13" t="inlineStr">
@@ -19452,16 +19395,16 @@
         </is>
       </c>
       <c r="F243" s="9" t="n">
-        <v>219</v>
+        <v>191</v>
       </c>
       <c r="G243" s="16" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B244" s="12" t="inlineStr">
@@ -19485,16 +19428,16 @@
         </is>
       </c>
       <c r="F244" s="6" t="n">
-        <v>140</v>
+        <v>191</v>
       </c>
       <c r="G244" s="15" t="n">
-        <v>-79</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="8" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B245" s="13" t="inlineStr">
@@ -19518,16 +19461,16 @@
         </is>
       </c>
       <c r="F245" s="9" t="n">
-        <v>177</v>
-      </c>
-      <c r="G245" s="16" t="n">
-        <v>37</v>
+        <v>191</v>
+      </c>
+      <c r="G245" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B246" s="12" t="inlineStr">
@@ -19551,16 +19494,16 @@
         </is>
       </c>
       <c r="F246" s="6" t="n">
-        <v>205</v>
-      </c>
-      <c r="G246" s="17" t="n">
-        <v>28</v>
+        <v>191</v>
+      </c>
+      <c r="G246" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B247" s="13" t="inlineStr">
@@ -19584,759 +19527,956 @@
         </is>
       </c>
       <c r="F247" s="9" t="n">
-        <v>152</v>
-      </c>
-      <c r="G247" s="14" t="n">
-        <v>-53</v>
-      </c>
-    </row>
-    <row r="249" ht="18" customHeight="1">
-      <c r="A249" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
-        </is>
+        <v>219</v>
+      </c>
+      <c r="G247" s="16" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B248" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C248" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D248" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E248" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F248" s="6" t="n">
+        <v>140</v>
+      </c>
+      <c r="G248" s="15" t="n">
+        <v>-79</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B249" s="13" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C249" s="8" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D249" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E249" s="8" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F249" s="9" t="n">
+        <v>177</v>
+      </c>
+      <c r="G249" s="16" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="5" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B250" s="12" t="inlineStr">
         <is>
-          <t>21:35_BRI_ret_BRI</t>
+          <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="C250" s="5" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D250" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E250" s="5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="F250" s="6" t="n">
-        <v>329</v>
-      </c>
-      <c r="G250" s="5" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
+        <v>205</v>
+      </c>
+      <c r="G250" s="17" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="8" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B251" s="13" t="inlineStr">
         <is>
-          <t>21:35_BRI_ret_BRI</t>
+          <t>21:30_IBE_ret_IBE</t>
         </is>
       </c>
       <c r="C251" s="8" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D251" s="8" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="E251" s="8" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="F251" s="9" t="n">
-        <v>280</v>
+        <v>152</v>
       </c>
       <c r="G251" s="14" t="n">
-        <v>-49</v>
+        <v>-53</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="5" t="inlineStr">
         <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B252" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="C252" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D252" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E252" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="F252" s="6" t="n">
+        <v>131</v>
+      </c>
+      <c r="G252" s="15" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="254" ht="18" customHeight="1">
+      <c r="A254" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Combination: 21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B255" s="12" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C255" s="5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D255" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E255" s="5" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F255" s="6" t="n">
+        <v>329</v>
+      </c>
+      <c r="G255" s="5" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B256" s="13" t="inlineStr">
+        <is>
+          <t>21:35_BRI_ret_BRI</t>
+        </is>
+      </c>
+      <c r="C256" s="8" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="D256" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="E256" s="8" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F256" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="G256" s="14" t="n">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="5" t="inlineStr">
+        <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B252" s="12" t="inlineStr">
+      <c r="B257" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C252" s="5" t="inlineStr">
+      <c r="C257" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D252" s="5" t="inlineStr">
+      <c r="D257" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E252" s="5" t="inlineStr">
+      <c r="E257" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F252" s="6" t="n">
+      <c r="F257" s="6" t="n">
         <v>294</v>
       </c>
-      <c r="G252" s="17" t="n">
+      <c r="G257" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="253">
-      <c r="A253" s="8" t="inlineStr">
+    <row r="258">
+      <c r="A258" s="8" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B253" s="13" t="inlineStr">
+      <c r="B258" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C253" s="8" t="inlineStr">
+      <c r="C258" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D253" s="8" t="inlineStr">
+      <c r="D258" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E253" s="8" t="inlineStr">
+      <c r="E258" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F253" s="9" t="n">
+      <c r="F258" s="9" t="n">
         <v>294</v>
       </c>
-      <c r="G253" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" s="5" t="inlineStr">
+      <c r="G258" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="5" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B254" s="12" t="inlineStr">
+      <c r="B259" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C254" s="5" t="inlineStr">
+      <c r="C259" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D254" s="5" t="inlineStr">
+      <c r="D259" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E254" s="5" t="inlineStr">
+      <c r="E259" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F254" s="6" t="n">
+      <c r="F259" s="6" t="n">
         <v>295</v>
       </c>
-      <c r="G254" s="17" t="n">
+      <c r="G259" s="17" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="255">
-      <c r="A255" s="8" t="inlineStr">
+    <row r="260">
+      <c r="A260" s="8" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B255" s="13" t="inlineStr">
+      <c r="B260" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C255" s="8" t="inlineStr">
+      <c r="C260" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D255" s="8" t="inlineStr">
+      <c r="D260" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E255" s="8" t="inlineStr">
+      <c r="E260" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F255" s="9" t="n">
+      <c r="F260" s="9" t="n">
         <v>269</v>
       </c>
-      <c r="G255" s="14" t="n">
+      <c r="G260" s="14" t="n">
         <v>-26</v>
       </c>
     </row>
-    <row r="256">
-      <c r="A256" s="5" t="inlineStr">
+    <row r="261">
+      <c r="A261" s="5" t="inlineStr">
         <is>
           <t>2026-07-26</t>
         </is>
       </c>
-      <c r="B256" s="12" t="inlineStr">
+      <c r="B261" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C256" s="5" t="inlineStr">
+      <c r="C261" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D256" s="5" t="inlineStr">
+      <c r="D261" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E256" s="5" t="inlineStr">
+      <c r="E261" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F256" s="6" t="n">
+      <c r="F261" s="6" t="n">
         <v>286</v>
       </c>
-      <c r="G256" s="17" t="n">
+      <c r="G261" s="17" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="257">
-      <c r="A257" s="8" t="inlineStr">
+    <row r="262">
+      <c r="A262" s="8" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B257" s="13" t="inlineStr">
+      <c r="B262" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C257" s="8" t="inlineStr">
+      <c r="C262" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D257" s="8" t="inlineStr">
+      <c r="D262" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E257" s="8" t="inlineStr">
+      <c r="E262" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F257" s="9" t="n">
+      <c r="F262" s="9" t="n">
         <v>286</v>
       </c>
-      <c r="G257" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="5" t="inlineStr">
+      <c r="G262" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="5" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B258" s="12" t="inlineStr">
+      <c r="B263" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C258" s="5" t="inlineStr">
+      <c r="C263" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D258" s="5" t="inlineStr">
+      <c r="D263" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E258" s="5" t="inlineStr">
+      <c r="E263" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F258" s="6" t="n">
+      <c r="F263" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="G258" s="17" t="n">
+      <c r="G263" s="17" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="259">
-      <c r="A259" s="8" t="inlineStr">
+    <row r="264">
+      <c r="A264" s="8" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B259" s="13" t="inlineStr">
+      <c r="B264" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C259" s="8" t="inlineStr">
+      <c r="C264" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D259" s="8" t="inlineStr">
+      <c r="D264" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E259" s="8" t="inlineStr">
+      <c r="E264" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F259" s="9" t="n">
+      <c r="F264" s="9" t="n">
         <v>325</v>
       </c>
-      <c r="G259" s="16" t="n">
+      <c r="G264" s="16" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="260">
-      <c r="A260" s="5" t="inlineStr">
+    <row r="265">
+      <c r="A265" s="5" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B260" s="12" t="inlineStr">
+      <c r="B265" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C260" s="5" t="inlineStr">
+      <c r="C265" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D260" s="5" t="inlineStr">
+      <c r="D265" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E260" s="5" t="inlineStr">
+      <c r="E265" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F260" s="6" t="n">
+      <c r="F265" s="6" t="n">
         <v>353</v>
       </c>
-      <c r="G260" s="17" t="n">
+      <c r="G265" s="17" t="n">
         <v>28</v>
       </c>
     </row>
-    <row r="261">
-      <c r="A261" s="8" t="inlineStr">
+    <row r="266">
+      <c r="A266" s="8" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="B261" s="13" t="inlineStr">
+      <c r="B266" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C261" s="8" t="inlineStr">
+      <c r="C266" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D261" s="8" t="inlineStr">
+      <c r="D266" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E261" s="8" t="inlineStr">
+      <c r="E266" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F261" s="9" t="n">
+      <c r="F266" s="9" t="n">
         <v>367</v>
       </c>
-      <c r="G261" s="16" t="n">
+      <c r="G266" s="16" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="262">
-      <c r="A262" s="5" t="inlineStr">
+    <row r="267">
+      <c r="A267" s="5" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B262" s="12" t="inlineStr">
+      <c r="B267" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C262" s="5" t="inlineStr">
+      <c r="C267" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D262" s="5" t="inlineStr">
+      <c r="D267" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E262" s="5" t="inlineStr">
+      <c r="E267" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F262" s="6" t="n">
+      <c r="F267" s="6" t="n">
         <v>353</v>
       </c>
-      <c r="G262" s="15" t="n">
+      <c r="G267" s="15" t="n">
         <v>-14</v>
       </c>
     </row>
-    <row r="263">
-      <c r="A263" s="8" t="inlineStr">
+    <row r="268">
+      <c r="A268" s="8" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B263" s="13" t="inlineStr">
+      <c r="B268" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C263" s="8" t="inlineStr">
+      <c r="C268" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D263" s="8" t="inlineStr">
+      <c r="D268" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E263" s="8" t="inlineStr">
+      <c r="E268" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F263" s="9" t="n">
+      <c r="F268" s="9" t="n">
         <v>346</v>
       </c>
-      <c r="G263" s="14" t="n">
+      <c r="G268" s="14" t="n">
         <v>-7</v>
       </c>
     </row>
-    <row r="264">
-      <c r="A264" s="5" t="inlineStr">
+    <row r="269">
+      <c r="A269" s="5" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B264" s="12" t="inlineStr">
+      <c r="B269" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C264" s="5" t="inlineStr">
+      <c r="C269" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D264" s="5" t="inlineStr">
+      <c r="D269" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E264" s="5" t="inlineStr">
+      <c r="E269" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F264" s="6" t="n">
+      <c r="F269" s="6" t="n">
         <v>537</v>
       </c>
-      <c r="G264" s="17" t="n">
+      <c r="G269" s="17" t="n">
         <v>191</v>
       </c>
     </row>
-    <row r="265">
-      <c r="A265" s="8" t="inlineStr">
+    <row r="270">
+      <c r="A270" s="8" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="B265" s="13" t="inlineStr">
+      <c r="B270" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C265" s="8" t="inlineStr">
+      <c r="C270" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D265" s="8" t="inlineStr">
+      <c r="D270" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E265" s="8" t="inlineStr">
+      <c r="E270" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F265" s="9" t="n">
+      <c r="F270" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="G265" s="16" t="n">
+      <c r="G270" s="16" t="n">
         <v>163</v>
       </c>
     </row>
-    <row r="266">
-      <c r="A266" s="5" t="inlineStr">
+    <row r="271">
+      <c r="A271" s="5" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="B266" s="12" t="inlineStr">
+      <c r="B271" s="12" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C266" s="5" t="inlineStr">
+      <c r="C271" s="5" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D266" s="5" t="inlineStr">
+      <c r="D271" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E266" s="5" t="inlineStr">
+      <c r="E271" s="5" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F266" s="6" t="n">
+      <c r="F271" s="6" t="n">
         <v>727</v>
       </c>
-      <c r="G266" s="17" t="n">
+      <c r="G271" s="17" t="n">
         <v>27</v>
       </c>
     </row>
-    <row r="267">
-      <c r="A267" s="8" t="inlineStr">
+    <row r="272">
+      <c r="A272" s="8" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="B267" s="13" t="inlineStr">
+      <c r="B272" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="C267" s="8" t="inlineStr">
+      <c r="C272" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="D267" s="8" t="inlineStr">
+      <c r="D272" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E267" s="8" t="inlineStr">
+      <c r="E272" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="F267" s="9" t="n">
+      <c r="F272" s="9" t="n">
         <v>757</v>
       </c>
-      <c r="G267" s="16" t="n">
+      <c r="G272" s="16" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="270" ht="20" customHeight="1">
-      <c r="A270" s="18" t="inlineStr">
+    <row r="275" ht="20" customHeight="1">
+      <c r="A275" s="18" t="inlineStr">
         <is>
           <t>Summary — Cheapest price seen per combination</t>
         </is>
       </c>
     </row>
-    <row r="271">
-      <c r="A271" s="3" t="inlineStr">
+    <row r="276">
+      <c r="A276" s="3" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="B271" s="3" t="inlineStr">
+      <c r="B276" s="3" t="inlineStr">
         <is>
           <t>Out time</t>
         </is>
       </c>
-      <c r="C271" s="3" t="inlineStr">
+      <c r="C276" s="3" t="inlineStr">
         <is>
           <t>Out airline</t>
         </is>
       </c>
-      <c r="D271" s="3" t="inlineStr">
+      <c r="D276" s="3" t="inlineStr">
         <is>
           <t>Ret airline</t>
         </is>
       </c>
-      <c r="E271" s="3" t="inlineStr">
+      <c r="E276" s="3" t="inlineStr">
         <is>
           <t>Min price</t>
         </is>
       </c>
-      <c r="F271" s="3" t="inlineStr">
+      <c r="F276" s="3" t="inlineStr">
         <is>
           <t>Max price</t>
         </is>
       </c>
-      <c r="G271" s="3" t="inlineStr">
+      <c r="G276" s="3" t="inlineStr">
         <is>
           <t>Avg price</t>
         </is>
       </c>
     </row>
-    <row r="272">
-      <c r="A272" s="12" t="inlineStr">
-        <is>
-          <t>17:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B272" s="5" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="C272" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D272" s="5" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E272" s="6" t="n">
+    <row r="277">
+      <c r="A277" s="12" t="inlineStr">
+        <is>
+          <t>17:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B277" s="5" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C277" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D277" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E277" s="6" t="n">
         <v>188</v>
       </c>
-      <c r="F272" s="6" t="n">
-        <v>309</v>
-      </c>
-      <c r="G272" s="6" t="n">
-        <v>250.96</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" s="13" t="inlineStr">
-        <is>
-          <t>21:30_IBE_ret_IBE</t>
-        </is>
-      </c>
-      <c r="B273" s="8" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C273" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="D273" s="8" t="inlineStr">
-        <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="E273" s="9" t="n">
-        <v>140</v>
-      </c>
-      <c r="F273" s="9" t="n">
+      <c r="F277" s="6" t="n">
+        <v>430</v>
+      </c>
+      <c r="G277" s="6" t="n">
+        <v>252.44</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="13" t="inlineStr">
+        <is>
+          <t>20:30_AIR_ret_AIR</t>
+        </is>
+      </c>
+      <c r="B278" s="8" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C278" s="8" t="inlineStr">
+        <is>
+          <t>Air France</t>
+        </is>
+      </c>
+      <c r="D278" s="8" t="inlineStr">
+        <is>
+          <t>Air France</t>
+        </is>
+      </c>
+      <c r="E278" s="9" t="n">
+        <v>547</v>
+      </c>
+      <c r="F278" s="9" t="n">
+        <v>547</v>
+      </c>
+      <c r="G278" s="9" t="n">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="12" t="inlineStr">
+        <is>
+          <t>21:30_IBE_ret_IBE</t>
+        </is>
+      </c>
+      <c r="B279" s="5" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C279" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="D279" s="5" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="E279" s="6" t="n">
+        <v>131</v>
+      </c>
+      <c r="F279" s="6" t="n">
         <v>256</v>
       </c>
-      <c r="G273" s="9" t="n">
-        <v>221.18</v>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" s="12" t="inlineStr">
+      <c r="G279" s="6" t="n">
+        <v>220.43</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="13" t="inlineStr">
         <is>
           <t>21:35_BRI_ret_BRI</t>
         </is>
       </c>
-      <c r="B274" s="5" t="inlineStr">
+      <c r="B280" s="8" t="inlineStr">
         <is>
           <t>21:35</t>
         </is>
       </c>
-      <c r="C274" s="5" t="inlineStr">
+      <c r="C280" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="D274" s="5" t="inlineStr">
+      <c r="D280" s="8" t="inlineStr">
         <is>
           <t>British Airways</t>
         </is>
       </c>
-      <c r="E274" s="6" t="n">
+      <c r="E280" s="9" t="n">
         <v>269</v>
       </c>
-      <c r="F274" s="6" t="n">
+      <c r="F280" s="9" t="n">
         <v>757</v>
       </c>
-      <c r="G274" s="6" t="n">
+      <c r="G280" s="9" t="n">
         <v>394.33</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="A254:G254"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A249:G249"/>
-    <mergeCell ref="A127:G127"/>
-    <mergeCell ref="A270:G270"/>
+    <mergeCell ref="A131:G131"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A275:G275"/>
+    <mergeCell ref="A128:G128"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>